<commit_message>
Add messages more Japanese information
</commit_message>
<xml_diff>
--- a/text-of-joker.cardpool.xlsx
+++ b/text-of-joker.cardpool.xlsx
@@ -2,13 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/78c39be24f0b20aa/ドキュメント/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{C6F0A1A7-64A3-47A6-82BD-5B1E68153299}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C699BC88-6DAB-453B-BBD1-B4D5776C06DC}"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7709F13D-D041-48AD-9F45-F91C5E8735D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{DC8CCAA9-C70A-4410-9BDB-26BCE8FF7367}"/>
   </bookViews>
@@ -4595,5 +4590,6 @@
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>